<commit_message>
Outreach status: add not-yet-contacted plants from Pietra list, Ally Nutra, PRL (28.10)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013pAYVPcDWTLeuLdwVsKmmQ
</commit_message>
<xml_diff>
--- a/suppliers_us/Aldera_outreach_status_2026-10-23.xlsx
+++ b/suppliers_us/Aldera_outreach_status_2026-10-23.xlsx
@@ -987,7 +987,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1314,6 +1314,316 @@
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Willings Nutraceutical</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Черри-Хилл, Нью-Джерси</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>856-424-9088</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>4-6 недель, срочно от 2 недель</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>есть</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Simpson Labs</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Валенсия, Калифорния</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>661-347-4348</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>капсулы, порошки, стики; органик, кошер, халяль</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>есть</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Evolve Contract Manufacturing</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Линдон, Юта</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>801-580-9151</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>капсулы, порошки, private label</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>есть</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>LaCore Nutraceuticals</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Ван-Алстайн, Техас</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>469-274-0106</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>капсулы, порошки</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>есть</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Wasatch Product Development</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Дрейпер, Юта</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>801-566-4449</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>крупный завод, от формулы до отправки</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>есть</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Ally Nutra</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Довер, Делавэр</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>888-720-5888</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>6 недель с гарантией $300/день, заказ от $15 000, стики</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>есть</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Premier Research Labs</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Остин, Техас</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>(800) 325-7734</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>программа private label для специалистов</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>есть</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Divine Design Manufacturing</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>нет данных (через Pietra)</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>заявляют самые короткие сроки</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>НЕТ: просить сертификат</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>We Do Private Label</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>нет данных (через Pietra)</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>минимум от 100 шт.</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>НЕТ: просить сертификат</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Smash Pharma</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Техас (через Pietra)</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>порошки, стики</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>НЕТ: просить сертификат</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>